<commit_message>
Complete FAPO Excel image data
</commit_message>
<xml_diff>
--- a/oferty/FAPO_Polska_katalog_kalkulacja_2026-05-25.xlsx
+++ b/oferty/FAPO_Polska_katalog_kalkulacja_2026-05-25.xlsx
@@ -2265,9 +2265,13 @@
           <t>https://fapomoto.pl/produkty/p0206-pz282510-front-stabilizer-sway-bar-end-links-for-honda-civic-12-15-mini-cooper-r56-06-13.html</t>
         </is>
       </c>
-      <c r="P16" s="19" t="inlineStr"/>
+      <c r="P16" s="21" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0764/7258/2395/files/PZ285210_3.jpg?v=1754383793</t>
+        </is>
+      </c>
       <c r="Q16" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
@@ -2569,9 +2573,13 @@
           <t>https://fapomoto.pl/produkty/p0209-pz293010-front-stabilizer-sway-bar-end-links-for-volkswagen-jetta-mk5-mk6-fwd-06-17.html</t>
         </is>
       </c>
-      <c r="P20" s="19" t="inlineStr"/>
+      <c r="P20" s="21" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0764/7258/2395/files/PZ292710_3_ba1d01b9-144b-4b81-a1f2-8836b07720f6.jpg?v=1756285583</t>
+        </is>
+      </c>
       <c r="Q20" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="13" t="inlineStr">
         <is>
@@ -8115,7 +8123,7 @@
         </is>
       </c>
       <c r="Q92" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R92" s="13" t="inlineStr">
         <is>
@@ -8192,7 +8200,7 @@
         </is>
       </c>
       <c r="Q93" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R93" s="16" t="inlineStr">
         <is>
@@ -10040,7 +10048,7 @@
         </is>
       </c>
       <c r="Q117" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R117" s="16" t="inlineStr">
         <is>
@@ -10117,7 +10125,7 @@
         </is>
       </c>
       <c r="Q118" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R118" s="13" t="inlineStr">
         <is>
@@ -10194,7 +10202,7 @@
         </is>
       </c>
       <c r="Q119" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R119" s="16" t="inlineStr">
         <is>
@@ -10502,7 +10510,7 @@
         </is>
       </c>
       <c r="Q123" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R123" s="16" t="inlineStr">
         <is>
@@ -11965,7 +11973,7 @@
         </is>
       </c>
       <c r="Q142" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R142" s="13" t="inlineStr">
         <is>
@@ -15199,7 +15207,7 @@
         </is>
       </c>
       <c r="Q184" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R184" s="13" t="inlineStr">
         <is>
@@ -16431,7 +16439,7 @@
         </is>
       </c>
       <c r="Q200" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R200" s="13" t="inlineStr">
         <is>
@@ -18818,7 +18826,7 @@
         </is>
       </c>
       <c r="Q231" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R231" s="16" t="inlineStr">
         <is>
@@ -19357,7 +19365,7 @@
         </is>
       </c>
       <c r="Q238" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R238" s="13" t="inlineStr">
         <is>
@@ -19434,7 +19442,7 @@
         </is>
       </c>
       <c r="Q239" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R239" s="16" t="inlineStr">
         <is>
@@ -22360,7 +22368,7 @@
         </is>
       </c>
       <c r="Q277" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R277" s="16" t="inlineStr">
         <is>
@@ -29906,7 +29914,7 @@
         </is>
       </c>
       <c r="Q375" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R375" s="16" t="inlineStr">
         <is>
@@ -30676,7 +30684,7 @@
         </is>
       </c>
       <c r="Q385" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R385" s="16" t="inlineStr">
         <is>
@@ -31831,7 +31839,7 @@
         </is>
       </c>
       <c r="Q400" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R400" s="13" t="inlineStr">
         <is>
@@ -32755,7 +32763,7 @@
         </is>
       </c>
       <c r="Q412" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R412" s="13" t="inlineStr">
         <is>
@@ -38453,7 +38461,7 @@
         </is>
       </c>
       <c r="Q486" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R486" s="13" t="inlineStr">
         <is>
@@ -38530,7 +38538,7 @@
         </is>
       </c>
       <c r="Q487" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R487" s="16" t="inlineStr">
         <is>
@@ -43067,9 +43075,13 @@
           <t>https://fapomoto.pl/produkty/p0316-pa291950-front-9-way-monotube-shocks-for-jeep-wrangler-jk-2007-2018-4-6-in-lift-pa291950.html</t>
         </is>
       </c>
-      <c r="P546" s="19" t="inlineStr"/>
+      <c r="P546" s="21" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0764/7258/2395/files/PA360650_1.jpg?v=1760599431</t>
+        </is>
+      </c>
       <c r="Q546" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R546" s="13" t="inlineStr">
         <is>
@@ -44757,9 +44769,13 @@
           <t>https://fapomoto.pl/produkty/p0317-pa491950-rear-9-way-monotube-shocks-for-jeep-wrangler-jk-2007-2018-4-6-in-lift-pa491950.html</t>
         </is>
       </c>
-      <c r="P568" s="19" t="inlineStr"/>
+      <c r="P568" s="21" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0764/7258/2395/files/PA660650_1.jpg?v=1760599919</t>
+        </is>
+      </c>
       <c r="Q568" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R568" s="13" t="inlineStr">
         <is>
@@ -44830,9 +44846,13 @@
           <t>https://fapomoto.pl/produkty/p0320-pa491950-pa291950-9-stage-full-set-4-6-in-lift-shocks-for-jeep-wrangler-jk-2007-2018.html</t>
         </is>
       </c>
-      <c r="P569" s="22" t="inlineStr"/>
+      <c r="P569" s="21" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0764/7258/2395/files/PA360650_PA660650_1.jpg?v=1760599919</t>
+        </is>
+      </c>
       <c r="Q569" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R569" s="16" t="inlineStr">
         <is>
@@ -46603,7 +46623,7 @@
         </is>
       </c>
       <c r="Q592" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R592" s="13" t="inlineStr">
         <is>
@@ -47065,7 +47085,7 @@
         </is>
       </c>
       <c r="Q598" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R598" s="13" t="inlineStr">
         <is>
@@ -47142,7 +47162,7 @@
         </is>
       </c>
       <c r="Q599" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R599" s="16" t="inlineStr">
         <is>
@@ -47450,7 +47470,7 @@
         </is>
       </c>
       <c r="Q603" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R603" s="16" t="inlineStr">
         <is>
@@ -47681,7 +47701,7 @@
         </is>
       </c>
       <c r="Q606" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R606" s="13" t="inlineStr">
         <is>
@@ -49580,1235 +49600,1240 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P50" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P51" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P52" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P53" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P59" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P63" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P65" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P67" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P69" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P70" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P71" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P72" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P73" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P74" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P75" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P76" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P77" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P78" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P79" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P80" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P81" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P82" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P83" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P84" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P85" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P86" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P87" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P88" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P89" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P90" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P91" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P92" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P93" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P94" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P95" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P96" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P97" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P98" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P99" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P100" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P101" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P102" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P103" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P104" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P105" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P106" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P107" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P108" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P109" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P110" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P111" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P112" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P113" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P114" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P115" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P116" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P117" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P118" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P119" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P120" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P121" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P122" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P123" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P124" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P125" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P126" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P127" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P128" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P129" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P130" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P131" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P132" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P133" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P134" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P135" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P136" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P137" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P138" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P139" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P140" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P141" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P142" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P143" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P144" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P145" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P146" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P147" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P148" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P149" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P150" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P151" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P152" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P153" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P154" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P155" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P156" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P157" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P158" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P159" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P160" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P161" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P162" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P163" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P164" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P165" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P166" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P167" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P168" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P169" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P170" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P171" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P172" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P173" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P174" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O175" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P175" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O176" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P176" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P177" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P178" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P179" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P180" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P181" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P182" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P183" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P184" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P185" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P186" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P187" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P188" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P189" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P190" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P191" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P192" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P193" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P194" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P195" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P196" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O197" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P197" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O198" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P198" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P199" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O200" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P200" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P201" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P202" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O203" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P203" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O204" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P204" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O205" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P205" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O206" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P206" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P207" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P208" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O209" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P209" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O210" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P210" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O211" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P211" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O212" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P212" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O213" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P213" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P214" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O215" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P215" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P216" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O217" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P217" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P218" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P219" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P220" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P221" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O222" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P222" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O223" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P223" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P224" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O225" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P225" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P226" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O227" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P227" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O228" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P228" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O229" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P229" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O230" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P230" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O231" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P231" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O232" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P232" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O233" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P233" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O234" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P234" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P235" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O236" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P236" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O237" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P237" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O238" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P238" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P239" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P240" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P241" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P242" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P243" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O244" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P244" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P245" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P246" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P247" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P248" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P249" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P250" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P251" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P252" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P253" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P254" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O255" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P255" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P256" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O257" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P257" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P258" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P259" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P260" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P261" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P262" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P263" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O264" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P264" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P265" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P266" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P267" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O268" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P268" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O269" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P269" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O270" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P270" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P271" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O272" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P272" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P273" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P274" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P275" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O276" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P276" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O277" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P277" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O278" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P278" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O279" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P279" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O280" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P280" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O281" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P281" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O282" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P282" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O283" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P283" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O284" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P284" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O285" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P285" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O286" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P286" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O287" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P287" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O288" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P288" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O289" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P289" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O290" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P290" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O291" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P291" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O292" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P292" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O293" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P293" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O294" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P294" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O295" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P295" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O296" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P296" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O297" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P297" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O298" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P298" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O299" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P299" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O300" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P300" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O301" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P301" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O302" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P302" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O303" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P303" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O304" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P304" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O305" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P305" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O306" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P306" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O307" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P307" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O308" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P308" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O309" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P309" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O310" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P310" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O311" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P311" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O312" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P312" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O313" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P313" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O314" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P314" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O315" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P315" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O316" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P316" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O317" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P317" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O318" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P318" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O319" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P319" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O320" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P320" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O321" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P321" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O322" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P322" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O323" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P323" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O324" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P324" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O325" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P325" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O326" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P326" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O327" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P327" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O328" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P328" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O329" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P329" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O330" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P330" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O331" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P331" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O332" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P332" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O333" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P333" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O334" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P334" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O335" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P335" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O336" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P336" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O337" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P337" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O338" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P338" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O339" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P339" r:id="rId674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O340" r:id="rId675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P340" r:id="rId676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O341" r:id="rId677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P341" r:id="rId678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O342" r:id="rId679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P342" r:id="rId680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O343" r:id="rId681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P343" r:id="rId682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O344" r:id="rId683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P344" r:id="rId684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O345" r:id="rId685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P345" r:id="rId686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O346" r:id="rId687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P346" r:id="rId688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O347" r:id="rId689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P347" r:id="rId690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O348" r:id="rId691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P348" r:id="rId692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O349" r:id="rId693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P349" r:id="rId694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O350" r:id="rId695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P350" r:id="rId696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O351" r:id="rId697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P351" r:id="rId698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O352" r:id="rId699"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P352" r:id="rId700"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O353" r:id="rId701"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P353" r:id="rId702"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O354" r:id="rId703"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P354" r:id="rId704"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O355" r:id="rId705"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P355" r:id="rId706"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O356" r:id="rId707"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P356" r:id="rId708"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O357" r:id="rId709"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P357" r:id="rId710"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O358" r:id="rId711"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P358" r:id="rId712"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O359" r:id="rId713"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P359" r:id="rId714"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O360" r:id="rId715"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P360" r:id="rId716"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O361" r:id="rId717"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P361" r:id="rId718"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O362" r:id="rId719"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P362" r:id="rId720"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O363" r:id="rId721"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P363" r:id="rId722"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O364" r:id="rId723"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P364" r:id="rId724"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O365" r:id="rId725"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P365" r:id="rId726"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O366" r:id="rId727"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P366" r:id="rId728"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O367" r:id="rId729"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P367" r:id="rId730"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O368" r:id="rId731"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P368" r:id="rId732"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O369" r:id="rId733"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P369" r:id="rId734"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O370" r:id="rId735"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P370" r:id="rId736"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O371" r:id="rId737"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P371" r:id="rId738"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O372" r:id="rId739"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P372" r:id="rId740"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O373" r:id="rId741"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P373" r:id="rId742"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O374" r:id="rId743"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P374" r:id="rId744"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O375" r:id="rId745"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P375" r:id="rId746"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O376" r:id="rId747"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P376" r:id="rId748"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O377" r:id="rId749"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P377" r:id="rId750"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O378" r:id="rId751"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P378" r:id="rId752"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O379" r:id="rId753"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P379" r:id="rId754"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O380" r:id="rId755"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P380" r:id="rId756"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O381" r:id="rId757"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P381" r:id="rId758"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O382" r:id="rId759"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P382" r:id="rId760"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O383" r:id="rId761"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P383" r:id="rId762"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O384" r:id="rId763"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P384" r:id="rId764"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O385" r:id="rId765"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P385" r:id="rId766"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O386" r:id="rId767"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P386" r:id="rId768"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O387" r:id="rId769"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P387" r:id="rId770"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O388" r:id="rId771"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P388" r:id="rId772"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O389" r:id="rId773"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P389" r:id="rId774"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O390" r:id="rId775"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P390" r:id="rId776"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O391" r:id="rId777"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P391" r:id="rId778"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O392" r:id="rId779"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P392" r:id="rId780"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O393" r:id="rId781"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P393" r:id="rId782"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O394" r:id="rId783"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P394" r:id="rId784"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O395" r:id="rId785"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P395" r:id="rId786"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O396" r:id="rId787"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P396" r:id="rId788"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O397" r:id="rId789"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P397" r:id="rId790"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O398" r:id="rId791"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P398" r:id="rId792"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O399" r:id="rId793"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P399" r:id="rId794"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O400" r:id="rId795"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P400" r:id="rId796"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O401" r:id="rId797"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P401" r:id="rId798"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O402" r:id="rId799"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P402" r:id="rId800"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O403" r:id="rId801"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P403" r:id="rId802"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O404" r:id="rId803"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P404" r:id="rId804"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O405" r:id="rId805"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P405" r:id="rId806"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O406" r:id="rId807"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P406" r:id="rId808"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O407" r:id="rId809"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P407" r:id="rId810"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O408" r:id="rId811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P408" r:id="rId812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O409" r:id="rId813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P409" r:id="rId814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O410" r:id="rId815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P410" r:id="rId816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O411" r:id="rId817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P411" r:id="rId818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O412" r:id="rId819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P412" r:id="rId820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O413" r:id="rId821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P413" r:id="rId822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O414" r:id="rId823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P414" r:id="rId824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O415" r:id="rId825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P415" r:id="rId826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O416" r:id="rId827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P416" r:id="rId828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O417" r:id="rId829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P417" r:id="rId830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O418" r:id="rId831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P418" r:id="rId832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O419" r:id="rId833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P419" r:id="rId834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O420" r:id="rId835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P420" r:id="rId836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O421" r:id="rId837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P421" r:id="rId838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O422" r:id="rId839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P422" r:id="rId840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O423" r:id="rId841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P423" r:id="rId842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O424" r:id="rId843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P424" r:id="rId844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O425" r:id="rId845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P425" r:id="rId846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O426" r:id="rId847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P426" r:id="rId848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O427" r:id="rId849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P427" r:id="rId850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O428" r:id="rId851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P428" r:id="rId852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O429" r:id="rId853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P429" r:id="rId854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O430" r:id="rId855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P430" r:id="rId856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O431" r:id="rId857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P431" r:id="rId858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O432" r:id="rId859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P432" r:id="rId860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O433" r:id="rId861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P433" r:id="rId862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O434" r:id="rId863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P434" r:id="rId864"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O435" r:id="rId865"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P435" r:id="rId866"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O436" r:id="rId867"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P436" r:id="rId868"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O437" r:id="rId869"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P437" r:id="rId870"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O438" r:id="rId871"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P438" r:id="rId872"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O439" r:id="rId873"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P439" r:id="rId874"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O440" r:id="rId875"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P440" r:id="rId876"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O441" r:id="rId877"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P441" r:id="rId878"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O442" r:id="rId879"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P442" r:id="rId880"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O443" r:id="rId881"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P443" r:id="rId882"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O444" r:id="rId883"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P444" r:id="rId884"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O445" r:id="rId885"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P445" r:id="rId886"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O446" r:id="rId887"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P446" r:id="rId888"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O447" r:id="rId889"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P447" r:id="rId890"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O448" r:id="rId891"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P448" r:id="rId892"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O449" r:id="rId893"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P449" r:id="rId894"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O450" r:id="rId895"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P450" r:id="rId896"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O451" r:id="rId897"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P451" r:id="rId898"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O452" r:id="rId899"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P452" r:id="rId900"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O453" r:id="rId901"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P453" r:id="rId902"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O454" r:id="rId903"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P454" r:id="rId904"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O455" r:id="rId905"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P455" r:id="rId906"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O456" r:id="rId907"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P456" r:id="rId908"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O457" r:id="rId909"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P457" r:id="rId910"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O458" r:id="rId911"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P458" r:id="rId912"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O459" r:id="rId913"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P459" r:id="rId914"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O460" r:id="rId915"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P460" r:id="rId916"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O461" r:id="rId917"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P461" r:id="rId918"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O462" r:id="rId919"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P462" r:id="rId920"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O463" r:id="rId921"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P463" r:id="rId922"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O464" r:id="rId923"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P464" r:id="rId924"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O465" r:id="rId925"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P465" r:id="rId926"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O466" r:id="rId927"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P466" r:id="rId928"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O467" r:id="rId929"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P467" r:id="rId930"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O468" r:id="rId931"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P468" r:id="rId932"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O469" r:id="rId933"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P469" r:id="rId934"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O470" r:id="rId935"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P470" r:id="rId936"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O471" r:id="rId937"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P471" r:id="rId938"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O472" r:id="rId939"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P472" r:id="rId940"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O473" r:id="rId941"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P473" r:id="rId942"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O474" r:id="rId943"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P474" r:id="rId944"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O475" r:id="rId945"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P475" r:id="rId946"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O476" r:id="rId947"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P476" r:id="rId948"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O477" r:id="rId949"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P477" r:id="rId950"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O478" r:id="rId951"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P478" r:id="rId952"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O479" r:id="rId953"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P479" r:id="rId954"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O480" r:id="rId955"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P480" r:id="rId956"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O481" r:id="rId957"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P481" r:id="rId958"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O482" r:id="rId959"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P482" r:id="rId960"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O483" r:id="rId961"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P483" r:id="rId962"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O484" r:id="rId963"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P484" r:id="rId964"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O485" r:id="rId965"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P485" r:id="rId966"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O486" r:id="rId967"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P486" r:id="rId968"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O487" r:id="rId969"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P487" r:id="rId970"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O488" r:id="rId971"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P488" r:id="rId972"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O489" r:id="rId973"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P489" r:id="rId974"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O490" r:id="rId975"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P490" r:id="rId976"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O491" r:id="rId977"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P491" r:id="rId978"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O492" r:id="rId979"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P492" r:id="rId980"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O493" r:id="rId981"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P493" r:id="rId982"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O494" r:id="rId983"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P494" r:id="rId984"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O495" r:id="rId985"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P495" r:id="rId986"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O496" r:id="rId987"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P496" r:id="rId988"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O497" r:id="rId989"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P497" r:id="rId990"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O498" r:id="rId991"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P498" r:id="rId992"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O499" r:id="rId993"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P499" r:id="rId994"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O500" r:id="rId995"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P500" r:id="rId996"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O501" r:id="rId997"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P501" r:id="rId998"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O502" r:id="rId999"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P502" r:id="rId1000"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O503" r:id="rId1001"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P503" r:id="rId1002"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O504" r:id="rId1003"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P504" r:id="rId1004"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O505" r:id="rId1005"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P505" r:id="rId1006"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O506" r:id="rId1007"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P506" r:id="rId1008"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O507" r:id="rId1009"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P507" r:id="rId1010"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O508" r:id="rId1011"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P508" r:id="rId1012"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O509" r:id="rId1013"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P509" r:id="rId1014"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O510" r:id="rId1015"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P510" r:id="rId1016"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O511" r:id="rId1017"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P511" r:id="rId1018"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O512" r:id="rId1019"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P512" r:id="rId1020"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O513" r:id="rId1021"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P513" r:id="rId1022"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O514" r:id="rId1023"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P514" r:id="rId1024"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O515" r:id="rId1025"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P515" r:id="rId1026"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O516" r:id="rId1027"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P516" r:id="rId1028"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O517" r:id="rId1029"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P517" r:id="rId1030"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O518" r:id="rId1031"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P518" r:id="rId1032"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O519" r:id="rId1033"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P519" r:id="rId1034"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O520" r:id="rId1035"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P520" r:id="rId1036"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O521" r:id="rId1037"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P521" r:id="rId1038"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O522" r:id="rId1039"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P522" r:id="rId1040"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O523" r:id="rId1041"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P523" r:id="rId1042"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O524" r:id="rId1043"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P524" r:id="rId1044"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O525" r:id="rId1045"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P525" r:id="rId1046"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O526" r:id="rId1047"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P526" r:id="rId1048"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O527" r:id="rId1049"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P527" r:id="rId1050"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O528" r:id="rId1051"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P528" r:id="rId1052"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O529" r:id="rId1053"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P529" r:id="rId1054"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O530" r:id="rId1055"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P530" r:id="rId1056"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O531" r:id="rId1057"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P531" r:id="rId1058"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O532" r:id="rId1059"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P532" r:id="rId1060"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O533" r:id="rId1061"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P533" r:id="rId1062"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O534" r:id="rId1063"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P534" r:id="rId1064"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O535" r:id="rId1065"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P535" r:id="rId1066"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O536" r:id="rId1067"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P536" r:id="rId1068"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O537" r:id="rId1069"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P537" r:id="rId1070"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O538" r:id="rId1071"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P538" r:id="rId1072"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O539" r:id="rId1073"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P539" r:id="rId1074"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O540" r:id="rId1075"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P540" r:id="rId1076"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O541" r:id="rId1077"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P541" r:id="rId1078"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O542" r:id="rId1079"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P542" r:id="rId1080"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O543" r:id="rId1081"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P543" r:id="rId1082"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O544" r:id="rId1083"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P544" r:id="rId1084"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O545" r:id="rId1085"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P545" r:id="rId1086"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O546" r:id="rId1087"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O547" r:id="rId1088"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P547" r:id="rId1089"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O548" r:id="rId1090"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P548" r:id="rId1091"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O549" r:id="rId1092"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P549" r:id="rId1093"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O550" r:id="rId1094"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P550" r:id="rId1095"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O551" r:id="rId1096"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P551" r:id="rId1097"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O552" r:id="rId1098"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P552" r:id="rId1099"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O553" r:id="rId1100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P553" r:id="rId1101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O554" r:id="rId1102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P554" r:id="rId1103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O555" r:id="rId1104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P555" r:id="rId1105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O556" r:id="rId1106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P556" r:id="rId1107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O557" r:id="rId1108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P557" r:id="rId1109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O558" r:id="rId1110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P558" r:id="rId1111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O559" r:id="rId1112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P559" r:id="rId1113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O560" r:id="rId1114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P560" r:id="rId1115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O561" r:id="rId1116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P561" r:id="rId1117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O562" r:id="rId1118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P562" r:id="rId1119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O563" r:id="rId1120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P563" r:id="rId1121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O564" r:id="rId1122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P564" r:id="rId1123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O565" r:id="rId1124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P565" r:id="rId1125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O566" r:id="rId1126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P566" r:id="rId1127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O567" r:id="rId1128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P567" r:id="rId1129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O568" r:id="rId1130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O569" r:id="rId1131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O570" r:id="rId1132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P570" r:id="rId1133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O571" r:id="rId1134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P571" r:id="rId1135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O572" r:id="rId1136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P572" r:id="rId1137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O573" r:id="rId1138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P573" r:id="rId1139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O574" r:id="rId1140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P574" r:id="rId1141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O575" r:id="rId1142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P575" r:id="rId1143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O576" r:id="rId1144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P576" r:id="rId1145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O577" r:id="rId1146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P577" r:id="rId1147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O578" r:id="rId1148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P578" r:id="rId1149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O579" r:id="rId1150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P579" r:id="rId1151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O580" r:id="rId1152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P580" r:id="rId1153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O581" r:id="rId1154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P581" r:id="rId1155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O582" r:id="rId1156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P582" r:id="rId1157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O583" r:id="rId1158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P583" r:id="rId1159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O584" r:id="rId1160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P584" r:id="rId1161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O585" r:id="rId1162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P585" r:id="rId1163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O586" r:id="rId1164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P586" r:id="rId1165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O587" r:id="rId1166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P587" r:id="rId1167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O588" r:id="rId1168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P588" r:id="rId1169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O589" r:id="rId1170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P589" r:id="rId1171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O590" r:id="rId1172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P590" r:id="rId1173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O591" r:id="rId1174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P591" r:id="rId1175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O592" r:id="rId1176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P592" r:id="rId1177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O593" r:id="rId1178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P593" r:id="rId1179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O594" r:id="rId1180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P594" r:id="rId1181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O595" r:id="rId1182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P595" r:id="rId1183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O596" r:id="rId1184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P596" r:id="rId1185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O597" r:id="rId1186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P597" r:id="rId1187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O598" r:id="rId1188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P598" r:id="rId1189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O599" r:id="rId1190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P599" r:id="rId1191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O600" r:id="rId1192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P600" r:id="rId1193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O601" r:id="rId1194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P601" r:id="rId1195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O602" r:id="rId1196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P602" r:id="rId1197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O603" r:id="rId1198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P603" r:id="rId1199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O604" r:id="rId1200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P604" r:id="rId1201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O605" r:id="rId1202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P605" r:id="rId1203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O606" r:id="rId1204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P606" r:id="rId1205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O607" r:id="rId1206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P607" r:id="rId1207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O608" r:id="rId1208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P608" r:id="rId1209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O609" r:id="rId1210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P609" r:id="rId1211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O610" r:id="rId1212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P610" r:id="rId1213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O611" r:id="rId1214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P611" r:id="rId1215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O612" r:id="rId1216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P612" r:id="rId1217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O613" r:id="rId1218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P613" r:id="rId1219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O614" r:id="rId1220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P614" r:id="rId1221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O615" r:id="rId1222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P615" r:id="rId1223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O616" r:id="rId1224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P616" r:id="rId1225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O617" r:id="rId1226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P617" r:id="rId1227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O618" r:id="rId1228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P618" r:id="rId1229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O619" r:id="rId1230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P619" r:id="rId1231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O620" r:id="rId1232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P620" r:id="rId1233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O621" r:id="rId1234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P621" r:id="rId1235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O622" r:id="rId1236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P622" r:id="rId1237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O623" r:id="rId1238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P623" r:id="rId1239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O624" r:id="rId1240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P624" r:id="rId1241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O625" r:id="rId1242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P625" r:id="rId1243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O626" r:id="rId1244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P626" r:id="rId1245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O627" r:id="rId1246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P627" r:id="rId1247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O628" r:id="rId1248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P628" r:id="rId1249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O629" r:id="rId1250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P629" r:id="rId1251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O630" r:id="rId1252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P630" r:id="rId1253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P51" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P59" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P63" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P65" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P67" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P69" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P70" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P71" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P72" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P73" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P74" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P75" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O76" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P76" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O77" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P77" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O78" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P78" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O79" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P79" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O80" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P80" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O81" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P81" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O82" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P82" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O83" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P83" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P84" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O85" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P85" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O86" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P86" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O87" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P87" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O88" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P88" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O89" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P89" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P90" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P91" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P92" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O93" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P93" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O94" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P94" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O95" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P95" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O96" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P96" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O97" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P97" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O98" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P98" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O99" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P99" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O100" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P100" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O101" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P101" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O102" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P102" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P103" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P104" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P105" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P106" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P107" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P108" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P109" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P110" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P111" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P112" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P113" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P114" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O115" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P115" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O116" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P116" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O117" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P117" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O118" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P118" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O119" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P119" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O120" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P120" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O121" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P121" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O122" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P122" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O123" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P123" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O124" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P124" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O125" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P125" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O126" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P126" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O127" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P127" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O128" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P128" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O129" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P129" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O130" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P130" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O131" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P131" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O132" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P132" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O133" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P133" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O134" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P134" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O135" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P135" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O136" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P136" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O137" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P137" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P138" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O139" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P139" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O140" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P140" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O141" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P141" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O142" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P142" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O143" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P143" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O144" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P144" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O145" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P145" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O146" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P146" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O147" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P147" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O148" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P148" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O149" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P149" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O150" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P150" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O151" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P151" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O152" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P152" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O153" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P153" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O154" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P154" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O155" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P155" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O156" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P156" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O157" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P157" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O158" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P158" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O159" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P159" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O160" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P160" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O161" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P161" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O162" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P162" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O163" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P163" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O164" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P164" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O165" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P165" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O166" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P166" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O167" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P167" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O168" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P168" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O169" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P169" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O170" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P170" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O171" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P171" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O172" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P172" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O173" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P173" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O174" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P174" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O175" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P175" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O176" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P176" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O177" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P177" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O178" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P178" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O179" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P179" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O180" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P180" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O181" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P181" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O182" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P182" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O183" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P183" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O184" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P184" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O185" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P185" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O186" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P186" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O187" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P187" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O188" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P188" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O189" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P189" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O190" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P190" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O191" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P191" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O192" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P192" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O193" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P193" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O194" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P194" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O195" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P195" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O196" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P196" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O197" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P197" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O198" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P198" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O199" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P199" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O200" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P200" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O201" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P201" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O202" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P202" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O203" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P203" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O204" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P204" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O205" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P205" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O206" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P206" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O207" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P207" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O208" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P208" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O209" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P209" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O210" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P210" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O211" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P211" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O212" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P212" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O213" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P213" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O214" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P214" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O215" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P215" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O216" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P216" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O217" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P217" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O218" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P218" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O219" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P219" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O220" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P220" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O221" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P221" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O222" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P222" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O223" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P223" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O224" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P224" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O225" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P225" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O226" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P226" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O227" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P227" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O228" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P228" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O229" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P229" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O230" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P230" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O231" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P231" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O232" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P232" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O233" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P233" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O234" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P234" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O235" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P235" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O236" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P236" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O237" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P237" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O238" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P238" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O239" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P239" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O240" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P240" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O241" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P241" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O242" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P242" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O243" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P243" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O244" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P244" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O245" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P245" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O246" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P246" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O247" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P247" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O248" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P248" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O249" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P249" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O250" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P250" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O251" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P251" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O252" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P252" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O253" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P253" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O254" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P254" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O255" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P255" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O256" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P256" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O257" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P257" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O258" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P258" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O259" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P259" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O260" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P260" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O261" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P261" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O262" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P262" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O263" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P263" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O264" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P264" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O265" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P265" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O266" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P266" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O267" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P267" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O268" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P268" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O269" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P269" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O270" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P270" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O271" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P271" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O272" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P272" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O273" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P273" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O274" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P274" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O275" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P275" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O276" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P276" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O277" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P277" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O278" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P278" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O279" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P279" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O280" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P280" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O281" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P281" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O282" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P282" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O283" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P283" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O284" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P284" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O285" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P285" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O286" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P286" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O287" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P287" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O288" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P288" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O289" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P289" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O290" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P290" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O291" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P291" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O292" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P292" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O293" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P293" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O294" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P294" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O295" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P295" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O296" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P296" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O297" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P297" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O298" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P298" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O299" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P299" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O300" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P300" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O301" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P301" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O302" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P302" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O303" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P303" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O304" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P304" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O305" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P305" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O306" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P306" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O307" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P307" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O308" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P308" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O309" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P309" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O310" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P310" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O311" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P311" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O312" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P312" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O313" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P313" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O314" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P314" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O315" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P315" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O316" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P316" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O317" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P317" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O318" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P318" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O319" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P319" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O320" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P320" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O321" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P321" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O322" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P322" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O323" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P323" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O324" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P324" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O325" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P325" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O326" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P326" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O327" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P327" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O328" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P328" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O329" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P329" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O330" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P330" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O331" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P331" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O332" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P332" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O333" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P333" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O334" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P334" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O335" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P335" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O336" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P336" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O337" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P337" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O338" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P338" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O339" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P339" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O340" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P340" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O341" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P341" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O342" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P342" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O343" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P343" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O344" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P344" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O345" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P345" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O346" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P346" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O347" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P347" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O348" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P348" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O349" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P349" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O350" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P350" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O351" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P351" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O352" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P352" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O353" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P353" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O354" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P354" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O355" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P355" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O356" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P356" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O357" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P357" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O358" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P358" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O359" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P359" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O360" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P360" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O361" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P361" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O362" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P362" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O363" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P363" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O364" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P364" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O365" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P365" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O366" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P366" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O367" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P367" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O368" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P368" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O369" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P369" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O370" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P370" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O371" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P371" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O372" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P372" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O373" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P373" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O374" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P374" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O375" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P375" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O376" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P376" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O377" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P377" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O378" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P378" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O379" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P379" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O380" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P380" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O381" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P381" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O382" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P382" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O383" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P383" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O384" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P384" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O385" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P385" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O386" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P386" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O387" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P387" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O388" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P388" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O389" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P389" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O390" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P390" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O391" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P391" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O392" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P392" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O393" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P393" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O394" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P394" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O395" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P395" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O396" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P396" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O397" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P397" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O398" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P398" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O399" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P399" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O400" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P400" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O401" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P401" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O402" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P402" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O403" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P403" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O404" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P404" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O405" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P405" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O406" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P406" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O407" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P407" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O408" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P408" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O409" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P409" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O410" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P410" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O411" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P411" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O412" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P412" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O413" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P413" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O414" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P414" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O415" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P415" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O416" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P416" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O417" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P417" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O418" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P418" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O419" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P419" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O420" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P420" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O421" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P421" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O422" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P422" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O423" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P423" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O424" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P424" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O425" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P425" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O426" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P426" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O427" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P427" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O428" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P428" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O429" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P429" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O430" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P430" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O431" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P431" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O432" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P432" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O433" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P433" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O434" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P434" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O435" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P435" r:id="rId868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O436" r:id="rId869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P436" r:id="rId870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O437" r:id="rId871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P437" r:id="rId872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O438" r:id="rId873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P438" r:id="rId874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O439" r:id="rId875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P439" r:id="rId876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O440" r:id="rId877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P440" r:id="rId878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O441" r:id="rId879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P441" r:id="rId880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O442" r:id="rId881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P442" r:id="rId882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O443" r:id="rId883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P443" r:id="rId884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O444" r:id="rId885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P444" r:id="rId886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O445" r:id="rId887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P445" r:id="rId888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O446" r:id="rId889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P446" r:id="rId890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O447" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P447" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O448" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P448" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O449" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P449" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O450" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P450" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O451" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P451" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O452" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P452" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O453" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P453" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O454" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P454" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O455" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P455" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O456" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P456" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O457" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P457" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O458" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P458" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O459" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P459" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O460" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P460" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O461" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P461" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O462" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P462" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O463" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P463" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O464" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P464" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O465" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P465" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O466" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P466" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O467" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P467" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O468" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P468" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O469" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P469" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O470" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P470" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O471" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P471" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O472" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P472" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O473" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P473" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O474" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P474" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O475" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P475" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O476" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P476" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O477" r:id="rId951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P477" r:id="rId952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O478" r:id="rId953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P478" r:id="rId954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O479" r:id="rId955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P479" r:id="rId956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O480" r:id="rId957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P480" r:id="rId958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O481" r:id="rId959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P481" r:id="rId960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O482" r:id="rId961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P482" r:id="rId962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O483" r:id="rId963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P483" r:id="rId964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O484" r:id="rId965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P484" r:id="rId966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O485" r:id="rId967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P485" r:id="rId968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O486" r:id="rId969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P486" r:id="rId970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O487" r:id="rId971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P487" r:id="rId972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O488" r:id="rId973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P488" r:id="rId974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O489" r:id="rId975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P489" r:id="rId976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O490" r:id="rId977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P490" r:id="rId978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O491" r:id="rId979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P491" r:id="rId980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O492" r:id="rId981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P492" r:id="rId982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O493" r:id="rId983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P493" r:id="rId984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O494" r:id="rId985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P494" r:id="rId986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O495" r:id="rId987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P495" r:id="rId988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O496" r:id="rId989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P496" r:id="rId990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O497" r:id="rId991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P497" r:id="rId992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O498" r:id="rId993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P498" r:id="rId994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O499" r:id="rId995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P499" r:id="rId996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O500" r:id="rId997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P500" r:id="rId998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O501" r:id="rId999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P501" r:id="rId1000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O502" r:id="rId1001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P502" r:id="rId1002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O503" r:id="rId1003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P503" r:id="rId1004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O504" r:id="rId1005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P504" r:id="rId1006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O505" r:id="rId1007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P505" r:id="rId1008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O506" r:id="rId1009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P506" r:id="rId1010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O507" r:id="rId1011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P507" r:id="rId1012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O508" r:id="rId1013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P508" r:id="rId1014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O509" r:id="rId1015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P509" r:id="rId1016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O510" r:id="rId1017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P510" r:id="rId1018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O511" r:id="rId1019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P511" r:id="rId1020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O512" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P512" r:id="rId1022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O513" r:id="rId1023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P513" r:id="rId1024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O514" r:id="rId1025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P514" r:id="rId1026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O515" r:id="rId1027"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P515" r:id="rId1028"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O516" r:id="rId1029"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P516" r:id="rId1030"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O517" r:id="rId1031"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P517" r:id="rId1032"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O518" r:id="rId1033"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P518" r:id="rId1034"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O519" r:id="rId1035"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P519" r:id="rId1036"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O520" r:id="rId1037"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P520" r:id="rId1038"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O521" r:id="rId1039"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P521" r:id="rId1040"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O522" r:id="rId1041"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P522" r:id="rId1042"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O523" r:id="rId1043"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P523" r:id="rId1044"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O524" r:id="rId1045"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P524" r:id="rId1046"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O525" r:id="rId1047"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P525" r:id="rId1048"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O526" r:id="rId1049"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P526" r:id="rId1050"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O527" r:id="rId1051"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P527" r:id="rId1052"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O528" r:id="rId1053"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P528" r:id="rId1054"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O529" r:id="rId1055"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P529" r:id="rId1056"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O530" r:id="rId1057"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P530" r:id="rId1058"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O531" r:id="rId1059"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P531" r:id="rId1060"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O532" r:id="rId1061"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P532" r:id="rId1062"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O533" r:id="rId1063"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P533" r:id="rId1064"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O534" r:id="rId1065"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P534" r:id="rId1066"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O535" r:id="rId1067"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P535" r:id="rId1068"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O536" r:id="rId1069"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P536" r:id="rId1070"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O537" r:id="rId1071"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P537" r:id="rId1072"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O538" r:id="rId1073"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P538" r:id="rId1074"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O539" r:id="rId1075"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P539" r:id="rId1076"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O540" r:id="rId1077"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P540" r:id="rId1078"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O541" r:id="rId1079"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P541" r:id="rId1080"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O542" r:id="rId1081"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P542" r:id="rId1082"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O543" r:id="rId1083"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P543" r:id="rId1084"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O544" r:id="rId1085"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P544" r:id="rId1086"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O545" r:id="rId1087"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P545" r:id="rId1088"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O546" r:id="rId1089"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P546" r:id="rId1090"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O547" r:id="rId1091"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P547" r:id="rId1092"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O548" r:id="rId1093"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P548" r:id="rId1094"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O549" r:id="rId1095"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P549" r:id="rId1096"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O550" r:id="rId1097"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P550" r:id="rId1098"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O551" r:id="rId1099"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P551" r:id="rId1100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O552" r:id="rId1101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P552" r:id="rId1102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O553" r:id="rId1103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P553" r:id="rId1104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O554" r:id="rId1105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P554" r:id="rId1106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O555" r:id="rId1107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P555" r:id="rId1108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O556" r:id="rId1109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P556" r:id="rId1110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O557" r:id="rId1111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P557" r:id="rId1112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O558" r:id="rId1113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P558" r:id="rId1114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O559" r:id="rId1115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P559" r:id="rId1116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O560" r:id="rId1117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P560" r:id="rId1118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O561" r:id="rId1119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P561" r:id="rId1120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O562" r:id="rId1121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P562" r:id="rId1122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O563" r:id="rId1123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P563" r:id="rId1124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O564" r:id="rId1125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P564" r:id="rId1126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O565" r:id="rId1127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P565" r:id="rId1128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O566" r:id="rId1129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P566" r:id="rId1130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O567" r:id="rId1131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P567" r:id="rId1132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O568" r:id="rId1133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P568" r:id="rId1134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O569" r:id="rId1135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P569" r:id="rId1136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O570" r:id="rId1137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P570" r:id="rId1138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O571" r:id="rId1139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P571" r:id="rId1140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O572" r:id="rId1141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P572" r:id="rId1142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O573" r:id="rId1143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P573" r:id="rId1144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O574" r:id="rId1145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P574" r:id="rId1146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O575" r:id="rId1147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P575" r:id="rId1148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O576" r:id="rId1149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P576" r:id="rId1150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O577" r:id="rId1151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P577" r:id="rId1152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O578" r:id="rId1153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P578" r:id="rId1154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O579" r:id="rId1155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P579" r:id="rId1156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O580" r:id="rId1157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P580" r:id="rId1158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O581" r:id="rId1159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P581" r:id="rId1160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O582" r:id="rId1161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P582" r:id="rId1162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O583" r:id="rId1163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P583" r:id="rId1164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O584" r:id="rId1165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P584" r:id="rId1166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O585" r:id="rId1167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P585" r:id="rId1168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O586" r:id="rId1169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P586" r:id="rId1170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O587" r:id="rId1171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P587" r:id="rId1172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O588" r:id="rId1173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P588" r:id="rId1174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O589" r:id="rId1175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P589" r:id="rId1176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O590" r:id="rId1177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P590" r:id="rId1178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O591" r:id="rId1179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P591" r:id="rId1180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O592" r:id="rId1181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P592" r:id="rId1182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O593" r:id="rId1183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P593" r:id="rId1184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O594" r:id="rId1185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P594" r:id="rId1186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O595" r:id="rId1187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P595" r:id="rId1188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O596" r:id="rId1189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P596" r:id="rId1190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O597" r:id="rId1191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P597" r:id="rId1192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O598" r:id="rId1193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P598" r:id="rId1194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O599" r:id="rId1195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P599" r:id="rId1196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O600" r:id="rId1197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P600" r:id="rId1198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O601" r:id="rId1199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P601" r:id="rId1200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O602" r:id="rId1201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P602" r:id="rId1202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O603" r:id="rId1203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P603" r:id="rId1204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O604" r:id="rId1205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P604" r:id="rId1206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O605" r:id="rId1207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P605" r:id="rId1208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O606" r:id="rId1209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P606" r:id="rId1210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O607" r:id="rId1211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P607" r:id="rId1212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O608" r:id="rId1213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P608" r:id="rId1214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O609" r:id="rId1215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P609" r:id="rId1216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O610" r:id="rId1217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P610" r:id="rId1218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O611" r:id="rId1219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P611" r:id="rId1220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O612" r:id="rId1221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P612" r:id="rId1222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O613" r:id="rId1223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P613" r:id="rId1224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O614" r:id="rId1225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P614" r:id="rId1226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O615" r:id="rId1227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P615" r:id="rId1228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O616" r:id="rId1229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P616" r:id="rId1230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O617" r:id="rId1231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P617" r:id="rId1232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O618" r:id="rId1233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P618" r:id="rId1234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O619" r:id="rId1235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P619" r:id="rId1236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O620" r:id="rId1237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P620" r:id="rId1238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O621" r:id="rId1239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P621" r:id="rId1240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O622" r:id="rId1241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P622" r:id="rId1242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O623" r:id="rId1243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P623" r:id="rId1244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O624" r:id="rId1245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P624" r:id="rId1246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O625" r:id="rId1247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P625" r:id="rId1248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O626" r:id="rId1249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P626" r:id="rId1250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O627" r:id="rId1251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P627" r:id="rId1252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O628" r:id="rId1253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P628" r:id="rId1254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O629" r:id="rId1255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P629" r:id="rId1256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O630" r:id="rId1257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P630" r:id="rId1258"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1254"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1259"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>